<commit_message>
Update cutoff data: AIIMS, All India, Deemed
</commit_message>
<xml_diff>
--- a/data/AIIMS_Cutoff.xlsx
+++ b/data/AIIMS_Cutoff.xlsx
@@ -1152,10 +1152,10 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>686</v>
+        <v>695</v>
       </c>
     </row>
     <row r="3">
@@ -1180,10 +1180,10 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>633</v>
+        <v>685</v>
       </c>
     </row>
     <row r="4">
@@ -1208,10 +1208,10 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>254</v>
+        <v>292</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>632</v>
+        <v>680</v>
       </c>
     </row>
     <row r="5">
@@ -1236,10 +1236,10 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>644</v>
+        <v>793</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>614</v>
+        <v>662</v>
       </c>
     </row>
     <row r="6">
@@ -1264,10 +1264,10 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1405</v>
+        <v>987</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>601</v>
+        <v>658</v>
       </c>
     </row>
     <row r="7">
@@ -1292,10 +1292,10 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>524</v>
+        <v>571</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>619</v>
+        <v>669</v>
       </c>
     </row>
     <row r="8">
@@ -1320,10 +1320,10 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1142</v>
+        <v>1084</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>604</v>
+        <v>656</v>
       </c>
     </row>
     <row r="9">
@@ -1348,10 +1348,10 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1582</v>
+        <v>1220</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>598</v>
+        <v>654</v>
       </c>
     </row>
     <row r="10">
@@ -1376,10 +1376,10 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>7030</v>
+        <v>7782</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>565</v>
+        <v>608</v>
       </c>
     </row>
     <row r="11">
@@ -1404,10 +1404,10 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>11713</v>
+        <v>8673</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>552</v>
+        <v>604</v>
       </c>
     </row>
     <row r="12">
@@ -1432,10 +1432,10 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>765</v>
+        <v>664</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>611</v>
+        <v>666</v>
       </c>
     </row>
     <row r="13">
@@ -1460,10 +1460,10 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>1017</v>
+        <v>1233</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>606</v>
+        <v>654</v>
       </c>
     </row>
     <row r="14">
@@ -1488,10 +1488,10 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1086</v>
+        <v>1660</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>605</v>
+        <v>647</v>
       </c>
     </row>
     <row r="15">
@@ -1516,10 +1516,10 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2010</v>
+        <v>5396</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>593</v>
+        <v>618</v>
       </c>
     </row>
     <row r="16">
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>14786</v>
+        <v>10926</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>545</v>
+        <v>597</v>
       </c>
     </row>
     <row r="17">
@@ -1572,10 +1572,10 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1798</v>
+        <v>344</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>595</v>
+        <v>677</v>
       </c>
     </row>
     <row r="18">
@@ -1600,10 +1600,10 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>2453</v>
+        <v>714</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>589</v>
+        <v>665</v>
       </c>
     </row>
     <row r="19">
@@ -1628,10 +1628,10 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>3066</v>
+        <v>879</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>584</v>
+        <v>660</v>
       </c>
     </row>
     <row r="20">
@@ -1656,10 +1656,10 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>19371</v>
+        <v>3941</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>538</v>
+        <v>627</v>
       </c>
     </row>
     <row r="21">
@@ -1684,10 +1684,10 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>42487</v>
+        <v>4457</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>510</v>
+        <v>623</v>
       </c>
     </row>
     <row r="22">
@@ -1712,10 +1712,10 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1376</v>
+        <v>1008</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>601</v>
+        <v>657</v>
       </c>
     </row>
     <row r="23">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>2016</v>
+        <v>1683</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>593</v>
+        <v>646</v>
       </c>
     </row>
     <row r="24">
@@ -1768,10 +1768,10 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>2631</v>
+        <v>2323</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>587</v>
+        <v>640</v>
       </c>
     </row>
     <row r="25">
@@ -1796,10 +1796,10 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>11751</v>
+        <v>12796</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>552</v>
+        <v>592</v>
       </c>
     </row>
     <row r="26">
@@ -1824,10 +1824,10 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>12960</v>
+        <v>16950</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>549</v>
+        <v>582</v>
       </c>
     </row>
     <row r="27">
@@ -1852,10 +1852,10 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>781</v>
+        <v>537</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>611</v>
+        <v>670</v>
       </c>
     </row>
     <row r="28">
@@ -1880,10 +1880,10 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>1104</v>
+        <v>979</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>605</v>
+        <v>658</v>
       </c>
     </row>
     <row r="29">
@@ -1908,10 +1908,10 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>1715</v>
+        <v>1089</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>595</v>
+        <v>656</v>
       </c>
     </row>
     <row r="30">
@@ -1936,10 +1936,10 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>7924</v>
+        <v>6429</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>562</v>
+        <v>613</v>
       </c>
     </row>
     <row r="31">
@@ -1964,10 +1964,10 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>7835</v>
+        <v>8532</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>562</v>
+        <v>605</v>
       </c>
     </row>
     <row r="32">
@@ -1992,10 +1992,10 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>1907</v>
+        <v>1593</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>594</v>
+        <v>648</v>
       </c>
     </row>
     <row r="33">
@@ -2020,10 +2020,10 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>2540</v>
+        <v>2054</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>588</v>
+        <v>642</v>
       </c>
     </row>
     <row r="34">
@@ -2048,10 +2048,10 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>3028</v>
+        <v>2675</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>584</v>
+        <v>636</v>
       </c>
     </row>
     <row r="35">
@@ -2076,10 +2076,10 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>17167</v>
+        <v>16709</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>541</v>
+        <v>583</v>
       </c>
     </row>
     <row r="36">
@@ -2104,10 +2104,10 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>30313</v>
+        <v>24984</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>523</v>
+        <v>567</v>
       </c>
     </row>
     <row r="37">
@@ -2132,10 +2132,10 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>891</v>
+        <v>792</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>609</v>
+        <v>662</v>
       </c>
     </row>
     <row r="38">
@@ -2160,10 +2160,10 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1377</v>
+        <v>1350</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>601</v>
+        <v>651</v>
       </c>
     </row>
     <row r="39">
@@ -2188,10 +2188,10 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>2923</v>
+        <v>1839</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>592</v>
+        <v>645</v>
       </c>
     </row>
     <row r="40">
@@ -2216,10 +2216,10 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>8697</v>
+        <v>8360</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>560</v>
+        <v>606</v>
       </c>
     </row>
     <row r="41">
@@ -2244,10 +2244,10 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>16192</v>
+        <v>13431</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>542</v>
+        <v>591</v>
       </c>
     </row>
     <row r="42">
@@ -2272,10 +2272,10 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>706</v>
+        <v>1314</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>614</v>
+        <v>652</v>
       </c>
     </row>
     <row r="43">
@@ -2300,10 +2300,10 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>2575</v>
+        <v>2079</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>588</v>
+        <v>642</v>
       </c>
     </row>
     <row r="44">
@@ -2328,10 +2328,10 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>2924</v>
+        <v>3021</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>585</v>
+        <v>634</v>
       </c>
     </row>
     <row r="45">
@@ -2356,10 +2356,10 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>15552</v>
+        <v>16901</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>544</v>
+        <v>582</v>
       </c>
     </row>
     <row r="46">
@@ -2384,10 +2384,10 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>31007</v>
+        <v>21776</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>521</v>
+        <v>573</v>
       </c>
     </row>
     <row r="47">
@@ -2412,10 +2412,10 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>1798</v>
+        <v>1630</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>595</v>
+        <v>647</v>
       </c>
     </row>
     <row r="48">
@@ -2440,10 +2440,10 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>2453</v>
+        <v>2190</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>589</v>
+        <v>641</v>
       </c>
     </row>
     <row r="49">
@@ -2468,10 +2468,10 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>3066</v>
+        <v>2910</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>584</v>
+        <v>635</v>
       </c>
     </row>
     <row r="50">
@@ -2496,10 +2496,10 @@
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>19371</v>
+        <v>18819</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>538</v>
+        <v>578</v>
       </c>
     </row>
     <row r="51">
@@ -2524,10 +2524,10 @@
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>42487</v>
+        <v>26664</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>510</v>
+        <v>565</v>
       </c>
     </row>
     <row r="52">
@@ -2552,10 +2552,10 @@
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>3586</v>
+        <v>3090</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>580</v>
+        <v>633</v>
       </c>
     </row>
     <row r="53">
@@ -2580,10 +2580,10 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>4463</v>
+        <v>3771</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>576</v>
+        <v>628</v>
       </c>
     </row>
     <row r="54">
@@ -2608,10 +2608,10 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>4672</v>
+        <v>4569</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>575</v>
+        <v>623</v>
       </c>
     </row>
     <row r="55">
@@ -2636,10 +2636,10 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>36168</v>
+        <v>25371</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>516</v>
+        <v>567</v>
       </c>
     </row>
     <row r="56">
@@ -2664,10 +2664,10 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>59983</v>
+        <v>40599</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>494</v>
+        <v>546</v>
       </c>
     </row>
     <row r="57">
@@ -2692,10 +2692,10 @@
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>2552</v>
+        <v>2114</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>588</v>
+        <v>642</v>
       </c>
     </row>
     <row r="58">
@@ -2720,10 +2720,10 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>3151</v>
+        <v>2443</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>583</v>
+        <v>639</v>
       </c>
     </row>
     <row r="59">
@@ -2748,10 +2748,10 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>3355</v>
+        <v>3085</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>582</v>
+        <v>633</v>
       </c>
     </row>
     <row r="60">
@@ -2776,10 +2776,10 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>26906</v>
+        <v>19159</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>527</v>
+        <v>578</v>
       </c>
     </row>
     <row r="61">
@@ -2804,10 +2804,10 @@
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>46911</v>
+        <v>33950</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>506</v>
+        <v>554</v>
       </c>
     </row>
     <row r="62">
@@ -2832,10 +2832,10 @@
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>2417</v>
+        <v>2188</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>589</v>
+        <v>641</v>
       </c>
     </row>
     <row r="63">
@@ -2860,10 +2860,10 @@
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>3861</v>
+        <v>3049</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>579</v>
+        <v>634</v>
       </c>
     </row>
     <row r="64">
@@ -2888,10 +2888,10 @@
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>4703</v>
+        <v>3955</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>574</v>
+        <v>627</v>
       </c>
     </row>
     <row r="65">
@@ -2916,10 +2916,10 @@
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>17680</v>
+        <v>18440</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>540</v>
+        <v>579</v>
       </c>
     </row>
     <row r="66">
@@ -2944,10 +2944,10 @@
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>58762</v>
+        <v>37522</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>495</v>
+        <v>550</v>
       </c>
     </row>
     <row r="67">
@@ -2972,10 +2972,10 @@
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>3284</v>
+        <v>2634</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>582</v>
+        <v>637</v>
       </c>
     </row>
     <row r="68">
@@ -3000,10 +3000,10 @@
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>3545</v>
+        <v>3160</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>580</v>
+        <v>632</v>
       </c>
     </row>
     <row r="69">
@@ -3028,10 +3028,10 @@
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>3918</v>
+        <v>3586</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>578</v>
+        <v>629</v>
       </c>
     </row>
     <row r="70">
@@ -3056,10 +3056,10 @@
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>33926</v>
+        <v>22455</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>519</v>
+        <v>572</v>
       </c>
     </row>
     <row r="71">
@@ -3084,10 +3084,10 @@
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>49630</v>
+        <v>35875</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>503</v>
+        <v>552</v>
       </c>
     </row>
     <row r="72">
@@ -3112,10 +3112,10 @@
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>1793</v>
+        <v>1705</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>595</v>
+        <v>646</v>
       </c>
     </row>
     <row r="73">
@@ -3140,10 +3140,10 @@
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>3191</v>
+        <v>2592</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>583</v>
+        <v>637</v>
       </c>
     </row>
     <row r="74">
@@ -3168,10 +3168,10 @@
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>4225</v>
+        <v>3180</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>577</v>
+        <v>632</v>
       </c>
     </row>
     <row r="75">
@@ -3196,10 +3196,10 @@
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>17480</v>
+        <v>17543</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>541</v>
+        <v>581</v>
       </c>
     </row>
     <row r="76">
@@ -3224,10 +3224,10 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>45033</v>
+        <v>28792</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>507</v>
+        <v>561</v>
       </c>
     </row>
     <row r="77">
@@ -3252,10 +3252,10 @@
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>3898</v>
+        <v>3327</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>578</v>
+        <v>631</v>
       </c>
     </row>
     <row r="78">
@@ -3280,10 +3280,10 @@
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>4314</v>
+        <v>3834</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>576</v>
+        <v>627</v>
       </c>
     </row>
     <row r="79">
@@ -3308,10 +3308,10 @@
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>4945</v>
+        <v>4748</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>573</v>
+        <v>622</v>
       </c>
     </row>
     <row r="80">
@@ -3336,10 +3336,10 @@
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>36367</v>
+        <v>27322</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>516</v>
+        <v>564</v>
       </c>
     </row>
     <row r="81">
@@ -3364,10 +3364,10 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>43200</v>
+        <v>34696</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>508</v>
+        <v>553</v>
       </c>
     </row>
     <row r="82">
@@ -3392,10 +3392,10 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>4016</v>
+        <v>2997</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>578</v>
+        <v>634</v>
       </c>
     </row>
     <row r="83">
@@ -3420,10 +3420,10 @@
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>4708</v>
+        <v>3823</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>574</v>
+        <v>628</v>
       </c>
     </row>
     <row r="84">
@@ -3448,10 +3448,10 @@
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>5463</v>
+        <v>4802</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>571</v>
+        <v>621</v>
       </c>
     </row>
     <row r="85">
@@ -3476,10 +3476,10 @@
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>32675</v>
+        <v>27539</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>520</v>
+        <v>563</v>
       </c>
     </row>
     <row r="86">
@@ -3504,10 +3504,10 @@
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>55652</v>
+        <v>37116</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>498</v>
+        <v>550</v>
       </c>
     </row>
     <row r="87">
@@ -3532,10 +3532,10 @@
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>2642</v>
+        <v>2039</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>587</v>
+        <v>642</v>
       </c>
     </row>
     <row r="88">
@@ -3560,10 +3560,10 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>3287</v>
+        <v>2892</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>582</v>
+        <v>635</v>
       </c>
     </row>
     <row r="89">
@@ -3588,10 +3588,10 @@
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>3215</v>
+        <v>2889</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>582</v>
+        <v>635</v>
       </c>
     </row>
     <row r="90">
@@ -3616,10 +3616,10 @@
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>30407</v>
+        <v>20222</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>523</v>
+        <v>576</v>
       </c>
     </row>
     <row r="91">
@@ -3644,10 +3644,10 @@
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>48673</v>
+        <v>31646</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>504</v>
+        <v>557</v>
       </c>
     </row>
     <row r="92">
@@ -3672,10 +3672,10 @@
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>2486</v>
+        <v>2260</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>589</v>
+        <v>640</v>
       </c>
     </row>
     <row r="93">
@@ -3700,10 +3700,10 @@
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>3153</v>
+        <v>2786</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>583</v>
+        <v>636</v>
       </c>
     </row>
     <row r="94">
@@ -3728,10 +3728,10 @@
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>3666</v>
+        <v>3287</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>580</v>
+        <v>632</v>
       </c>
     </row>
     <row r="95">
@@ -3756,10 +3756,10 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>24786</v>
+        <v>20129</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>530</v>
+        <v>576</v>
       </c>
     </row>
     <row r="96">
@@ -3784,10 +3784,10 @@
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>41195</v>
+        <v>30805</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>511</v>
+        <v>559</v>
       </c>
     </row>
     <row r="97">
@@ -3812,10 +3812,10 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>5394</v>
+        <v>3421</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>571</v>
+        <v>630</v>
       </c>
     </row>
     <row r="98">
@@ -3840,10 +3840,10 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>6456</v>
+        <v>4281</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>567</v>
+        <v>625</v>
       </c>
     </row>
     <row r="99">
@@ -3868,10 +3868,10 @@
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>7417</v>
+        <v>5416</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>564</v>
+        <v>618</v>
       </c>
     </row>
     <row r="100">
@@ -3896,10 +3896,10 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>43997</v>
+        <v>27253</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>508</v>
+        <v>564</v>
       </c>
     </row>
     <row r="101">
@@ -3924,10 +3924,10 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>63398</v>
+        <v>44940</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>492</v>
+        <v>541</v>
       </c>
     </row>
     <row r="102">
@@ -3952,10 +3952,10 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>268965</v>
+        <v>225122</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>372</v>
+        <v>421</v>
       </c>
     </row>
     <row r="103">
@@ -3980,10 +3980,10 @@
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>174486</v>
+        <v>211861</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>420</v>
+        <v>427</v>
       </c>
     </row>
     <row r="104">
@@ -4008,10 +4008,10 @@
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>536109</v>
+        <v>470951</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>270</v>
+        <v>334</v>
       </c>
     </row>
     <row r="105">
@@ -4036,10 +4036,10 @@
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>330044</v>
+        <v>284684</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>345</v>
+        <v>395</v>
       </c>
     </row>
     <row r="106">
@@ -4064,10 +4064,10 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>241346</v>
+        <v>205434</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>385</v>
+        <v>430</v>
       </c>
     </row>
     <row r="107">
@@ -4092,10 +4092,10 @@
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>486740</v>
+        <v>386020</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>286</v>
+        <v>359</v>
       </c>
     </row>
     <row r="108">
@@ -4120,10 +4120,10 @@
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>340348</v>
+        <v>300462</v>
       </c>
       <c r="F108" s="2" t="n">
-        <v>341</v>
+        <v>389</v>
       </c>
     </row>
     <row r="109">
@@ -4148,10 +4148,10 @@
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>309667</v>
+        <v>189156</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>354</v>
+        <v>438</v>
       </c>
     </row>
     <row r="110">
@@ -4176,10 +4176,10 @@
         </is>
       </c>
       <c r="E110" s="2" t="n">
-        <v>730492</v>
+        <v>603010</v>
       </c>
       <c r="F110" s="2" t="n">
-        <v>217</v>
+        <v>298</v>
       </c>
     </row>
     <row r="111">
@@ -4204,10 +4204,10 @@
         </is>
       </c>
       <c r="E111" s="2" t="n">
-        <v>440047</v>
+        <v>388651</v>
       </c>
       <c r="F111" s="2" t="n">
-        <v>302</v>
+        <v>358</v>
       </c>
     </row>
     <row r="112">
@@ -4232,10 +4232,10 @@
         </is>
       </c>
       <c r="E112" s="2" t="n">
-        <v>354680</v>
+        <v>306676</v>
       </c>
       <c r="F112" s="2" t="n">
-        <v>335</v>
+        <v>387</v>
       </c>
     </row>
     <row r="113">
@@ -4260,10 +4260,10 @@
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>221837</v>
+        <v>239506</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>395</v>
+        <v>414</v>
       </c>
     </row>
     <row r="114">
@@ -4288,10 +4288,10 @@
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>518444</v>
+        <v>653328</v>
       </c>
       <c r="F114" s="2" t="n">
-        <v>277</v>
+        <v>286</v>
       </c>
     </row>
     <row r="115">
@@ -4316,10 +4316,10 @@
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>770273</v>
+        <v>490090</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>208</v>
+        <v>328</v>
       </c>
     </row>
     <row r="116">
@@ -4372,10 +4372,10 @@
         </is>
       </c>
       <c r="E117" s="2" t="n">
-        <v>401069</v>
+        <v>121006</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>316</v>
+        <v>478</v>
       </c>
     </row>
     <row r="118">
@@ -4400,10 +4400,10 @@
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>279531</v>
+        <v>94109</v>
       </c>
       <c r="F118" s="2" t="n">
-        <v>367</v>
+        <v>497</v>
       </c>
     </row>
     <row r="119">
@@ -4428,10 +4428,10 @@
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>630186</v>
+        <v>327534</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>243</v>
+        <v>379</v>
       </c>
     </row>
     <row r="120">
@@ -4484,10 +4484,10 @@
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>321581</v>
+        <v>269496</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>349</v>
+        <v>401</v>
       </c>
     </row>
     <row r="122">
@@ -4512,10 +4512,10 @@
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>229985</v>
+        <v>227773</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>391</v>
+        <v>420</v>
       </c>
     </row>
     <row r="123">
@@ -4568,10 +4568,10 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>241313</v>
+        <v>207083</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>385</v>
+        <v>429</v>
       </c>
     </row>
     <row r="125">
@@ -4596,10 +4596,10 @@
         </is>
       </c>
       <c r="E125" s="2" t="n">
-        <v>22426</v>
+        <v>37101</v>
       </c>
       <c r="F125" s="2" t="n">
-        <v>533</v>
+        <v>550</v>
       </c>
     </row>
     <row r="126">
@@ -4708,10 +4708,10 @@
         </is>
       </c>
       <c r="E129" s="2" t="n">
-        <v>258759</v>
+        <v>201937</v>
       </c>
       <c r="F129" s="2" t="n">
-        <v>377</v>
+        <v>432</v>
       </c>
     </row>
     <row r="130">
@@ -4736,10 +4736,10 @@
         </is>
       </c>
       <c r="E130" s="2" t="n">
-        <v>221694</v>
+        <v>88048</v>
       </c>
       <c r="F130" s="2" t="n">
-        <v>395</v>
+        <v>502</v>
       </c>
     </row>
     <row r="131">
@@ -4764,10 +4764,10 @@
         </is>
       </c>
       <c r="E131" s="2" t="n">
-        <v>225964</v>
+        <v>365084</v>
       </c>
       <c r="F131" s="2" t="n">
-        <v>393</v>
+        <v>366</v>
       </c>
     </row>
     <row r="132">
@@ -4792,10 +4792,10 @@
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>376997</v>
+        <v>295349</v>
       </c>
       <c r="F132" s="2" t="n">
-        <v>326</v>
+        <v>391</v>
       </c>
     </row>
     <row r="133">
@@ -4820,10 +4820,10 @@
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>305719</v>
+        <v>256215</v>
       </c>
       <c r="F133" s="2" t="n">
-        <v>356</v>
+        <v>407</v>
       </c>
     </row>
     <row r="134">
@@ -4848,10 +4848,10 @@
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>534447</v>
+        <v>485836</v>
       </c>
       <c r="F134" s="2" t="n">
-        <v>271</v>
+        <v>329</v>
       </c>
     </row>
     <row r="135">
@@ -4876,10 +4876,10 @@
         </is>
       </c>
       <c r="E135" s="2" t="n">
-        <v>396329</v>
+        <v>189449</v>
       </c>
       <c r="F135" s="2" t="n">
-        <v>318</v>
+        <v>438</v>
       </c>
     </row>
     <row r="136">
@@ -4904,10 +4904,10 @@
         </is>
       </c>
       <c r="E136" s="2" t="n">
-        <v>338406</v>
+        <v>133375</v>
       </c>
       <c r="F136" s="2" t="n">
-        <v>341</v>
+        <v>470</v>
       </c>
     </row>
     <row r="137">
@@ -4932,10 +4932,10 @@
         </is>
       </c>
       <c r="E137" s="2" t="n">
-        <v>294578</v>
+        <v>110199</v>
       </c>
       <c r="F137" s="2" t="n">
-        <v>361</v>
+        <v>485</v>
       </c>
     </row>
     <row r="138">
@@ -4960,10 +4960,10 @@
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>596639</v>
+        <v>488861</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>252</v>
+        <v>329</v>
       </c>
     </row>
     <row r="139">
@@ -5016,10 +5016,10 @@
         </is>
       </c>
       <c r="E140" s="2" t="n">
-        <v>98647</v>
+        <v>144446</v>
       </c>
       <c r="F140" s="2" t="n">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="141">
@@ -5044,10 +5044,10 @@
         </is>
       </c>
       <c r="E141" s="2" t="n">
-        <v>87801</v>
+        <v>49241</v>
       </c>
       <c r="F141" s="2" t="n">
-        <v>473</v>
+        <v>536</v>
       </c>
     </row>
     <row r="142">
@@ -5072,10 +5072,10 @@
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>234585</v>
+        <v>246013</v>
       </c>
       <c r="F142" s="2" t="n">
-        <v>389</v>
+        <v>411</v>
       </c>
     </row>
     <row r="143">
@@ -5156,10 +5156,10 @@
         </is>
       </c>
       <c r="E145" s="2" t="n">
-        <v>386570</v>
+        <v>292473</v>
       </c>
       <c r="F145" s="2" t="n">
-        <v>322</v>
+        <v>392</v>
       </c>
     </row>
     <row r="146">
@@ -5184,10 +5184,10 @@
         </is>
       </c>
       <c r="E146" s="2" t="n">
-        <v>262176</v>
+        <v>207392</v>
       </c>
       <c r="F146" s="2" t="n">
-        <v>375</v>
+        <v>429</v>
       </c>
     </row>
     <row r="147">
@@ -5296,10 +5296,10 @@
         </is>
       </c>
       <c r="E150" s="2" t="n">
-        <v>190373</v>
+        <v>167218</v>
       </c>
       <c r="F150" s="2" t="n">
-        <v>411</v>
+        <v>450</v>
       </c>
     </row>
     <row r="151">
@@ -5324,10 +5324,10 @@
         </is>
       </c>
       <c r="E151" s="2" t="n">
-        <v>339955</v>
+        <v>175335</v>
       </c>
       <c r="F151" s="2" t="n">
-        <v>341</v>
+        <v>446</v>
       </c>
     </row>
     <row r="152">
@@ -5352,10 +5352,10 @@
         </is>
       </c>
       <c r="E152" s="2" t="n">
-        <v>168613</v>
+        <v>178444</v>
       </c>
       <c r="F152" s="2" t="n">
-        <v>423</v>
+        <v>444</v>
       </c>
     </row>
     <row r="153">
@@ -5380,10 +5380,10 @@
         </is>
       </c>
       <c r="E153" s="2" t="n">
-        <v>137288</v>
+        <v>83566</v>
       </c>
       <c r="F153" s="2" t="n">
-        <v>442</v>
+        <v>505</v>
       </c>
     </row>
     <row r="154">
@@ -5408,10 +5408,10 @@
         </is>
       </c>
       <c r="E154" s="2" t="n">
-        <v>197744</v>
+        <v>287572</v>
       </c>
       <c r="F154" s="2" t="n">
-        <v>408</v>
+        <v>394</v>
       </c>
     </row>
     <row r="155">
@@ -5436,10 +5436,10 @@
         </is>
       </c>
       <c r="E155" s="2" t="n">
-        <v>31622</v>
+        <v>20015</v>
       </c>
       <c r="F155" s="2" t="n">
-        <v>521</v>
+        <v>576</v>
       </c>
     </row>
     <row r="156">
@@ -5464,10 +5464,10 @@
         </is>
       </c>
       <c r="E156" s="2" t="n">
-        <v>4801</v>
+        <v>5866</v>
       </c>
       <c r="F156" s="2" t="n">
-        <v>574</v>
+        <v>616</v>
       </c>
     </row>
     <row r="157">
@@ -5520,10 +5520,10 @@
         </is>
       </c>
       <c r="E158" s="2" t="n">
-        <v>324957</v>
+        <v>219399</v>
       </c>
       <c r="F158" s="2" t="n">
-        <v>347</v>
+        <v>423</v>
       </c>
     </row>
     <row r="159">
@@ -5548,10 +5548,10 @@
         </is>
       </c>
       <c r="E159" s="2" t="n">
-        <v>221737</v>
+        <v>210581</v>
       </c>
       <c r="F159" s="2" t="n">
-        <v>395</v>
+        <v>428</v>
       </c>
     </row>
     <row r="160">
@@ -5576,10 +5576,10 @@
         </is>
       </c>
       <c r="E160" s="2" t="n">
-        <v>436764</v>
+        <v>404611</v>
       </c>
       <c r="F160" s="2" t="n">
-        <v>303</v>
+        <v>353</v>
       </c>
     </row>
     <row r="161">
@@ -5632,10 +5632,10 @@
         </is>
       </c>
       <c r="E162" s="2" t="n">
-        <v>354913</v>
+        <v>245682</v>
       </c>
       <c r="F162" s="2" t="n">
-        <v>335</v>
+        <v>411</v>
       </c>
     </row>
     <row r="163">
@@ -5660,10 +5660,10 @@
         </is>
       </c>
       <c r="E163" s="2" t="n">
-        <v>327221</v>
+        <v>230014</v>
       </c>
       <c r="F163" s="2" t="n">
-        <v>346</v>
+        <v>419</v>
       </c>
     </row>
     <row r="164">
@@ -5688,10 +5688,10 @@
         </is>
       </c>
       <c r="E164" s="2" t="n">
-        <v>376229</v>
+        <v>528896</v>
       </c>
       <c r="F164" s="2" t="n">
-        <v>326</v>
+        <v>318</v>
       </c>
     </row>
     <row r="165">
@@ -5716,10 +5716,10 @@
         </is>
       </c>
       <c r="E165" s="2" t="n">
-        <v>1057165</v>
+        <v>485894</v>
       </c>
       <c r="F165" s="2" t="n">
-        <v>151</v>
+        <v>329</v>
       </c>
     </row>
     <row r="166">
@@ -5772,10 +5772,10 @@
         </is>
       </c>
       <c r="E167" s="2" t="n">
-        <v>306492</v>
+        <v>195831</v>
       </c>
       <c r="F167" s="2" t="n">
-        <v>355</v>
+        <v>435</v>
       </c>
     </row>
     <row r="168">
@@ -5800,10 +5800,10 @@
         </is>
       </c>
       <c r="E168" s="2" t="n">
-        <v>194869</v>
+        <v>189092</v>
       </c>
       <c r="F168" s="2" t="n">
-        <v>409</v>
+        <v>438</v>
       </c>
     </row>
     <row r="169">
@@ -5828,10 +5828,10 @@
         </is>
       </c>
       <c r="E169" s="2" t="n">
-        <v>230742</v>
+        <v>319126</v>
       </c>
       <c r="F169" s="2" t="n">
-        <v>391</v>
+        <v>382</v>
       </c>
     </row>
     <row r="170">
@@ -5856,10 +5856,10 @@
         </is>
       </c>
       <c r="E170" s="2" t="n">
-        <v>161370</v>
+        <v>84424</v>
       </c>
       <c r="F170" s="2" t="n">
-        <v>427</v>
+        <v>504</v>
       </c>
     </row>
     <row r="171">
@@ -5884,10 +5884,10 @@
         </is>
       </c>
       <c r="E171" s="2" t="n">
-        <v>147945</v>
+        <v>60079</v>
       </c>
       <c r="F171" s="2" t="n">
-        <v>435</v>
+        <v>525</v>
       </c>
     </row>
     <row r="172">
@@ -5912,10 +5912,10 @@
         </is>
       </c>
       <c r="E172" s="2" t="n">
-        <v>119885</v>
+        <v>143304</v>
       </c>
       <c r="F172" s="2" t="n">
-        <v>452</v>
+        <v>464</v>
       </c>
     </row>
     <row r="173">
@@ -5940,10 +5940,10 @@
         </is>
       </c>
       <c r="E173" s="2" t="n">
-        <v>116547</v>
+        <v>151227</v>
       </c>
       <c r="F173" s="2" t="n">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="174">
@@ -5968,10 +5968,10 @@
         </is>
       </c>
       <c r="E174" s="2" t="n">
-        <v>116405</v>
+        <v>103992</v>
       </c>
       <c r="F174" s="2" t="n">
-        <v>454</v>
+        <v>490</v>
       </c>
     </row>
     <row r="175">
@@ -5996,10 +5996,10 @@
         </is>
       </c>
       <c r="E175" s="2" t="n">
-        <v>261657</v>
+        <v>156322</v>
       </c>
       <c r="F175" s="2" t="n">
-        <v>376</v>
+        <v>456</v>
       </c>
     </row>
     <row r="176">
@@ -6024,10 +6024,10 @@
         </is>
       </c>
       <c r="E176" s="2" t="n">
-        <v>636315</v>
+        <v>457225</v>
       </c>
       <c r="F176" s="2" t="n">
-        <v>241</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>